<commit_message>
Update data package at: 2026-09-25T20:13:57Z
</commit_message>
<xml_diff>
--- a/data/dados_sigplan_2027/indicadores_planejamento.xlsx
+++ b/data/dados_sigplan_2027/indicadores_planejamento.xlsx
@@ -645,7 +645,7 @@
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
       <c r="X2" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y2" t="b">
         <v>0</v>
@@ -737,7 +737,7 @@
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
       <c r="X3" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y3" t="b">
         <v>0</v>
@@ -829,7 +829,7 @@
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
       <c r="X4" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y4" t="b">
         <v>1</v>
@@ -921,7 +921,7 @@
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr"/>
       <c r="X5" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y5" t="b">
         <v>1</v>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="W6" t="inlineStr"/>
       <c r="X6" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y6" t="b">
         <v>0</v>
@@ -1109,7 +1109,7 @@
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
       <c r="X7" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y7" t="b">
         <v>0</v>
@@ -1201,7 +1201,7 @@
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
       <c r="X8" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y8" t="b">
         <v>0</v>
@@ -1293,7 +1293,7 @@
         </is>
       </c>
       <c r="X9" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y9" t="b">
         <v>0</v>
@@ -1385,7 +1385,7 @@
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
       <c r="X10" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y10" t="b">
         <v>0</v>
@@ -1477,7 +1477,7 @@
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
       <c r="X11" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y11" t="b">
         <v>0</v>
@@ -1540,7 +1540,9 @@
       <c r="O12" t="b">
         <v>0</v>
       </c>
-      <c r="P12" t="inlineStr"/>
+      <c r="P12" t="n">
+        <v>714118</v>
+      </c>
       <c r="Q12" t="b">
         <v>0</v>
       </c>
@@ -1567,7 +1569,7 @@
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
       <c r="X12" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y12" t="b">
         <v>0</v>
@@ -1659,7 +1661,7 @@
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr"/>
       <c r="X13" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y13" t="b">
         <v>0</v>
@@ -1751,7 +1753,7 @@
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
       <c r="X14" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y14" t="b">
         <v>0</v>
@@ -1843,7 +1845,7 @@
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
       <c r="X15" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y15" t="b">
         <v>1</v>
@@ -1935,7 +1937,7 @@
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
       <c r="X16" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y16" t="b">
         <v>0</v>
@@ -2027,7 +2029,7 @@
       <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
       <c r="X17" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y17" t="b">
         <v>0</v>
@@ -2119,7 +2121,7 @@
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr"/>
       <c r="X18" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y18" t="b">
         <v>0</v>
@@ -2211,7 +2213,7 @@
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
       <c r="X19" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y19" t="b">
         <v>0</v>
@@ -2303,7 +2305,7 @@
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr"/>
       <c r="X20" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y20" t="b">
         <v>0</v>
@@ -2395,7 +2397,7 @@
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
       <c r="X21" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y21" t="b">
         <v>0</v>
@@ -2487,7 +2489,7 @@
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr"/>
       <c r="X22" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y22" t="b">
         <v>0</v>
@@ -2579,7 +2581,7 @@
       <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr"/>
       <c r="X23" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y23" t="b">
         <v>0</v>
@@ -2669,7 +2671,7 @@
         </is>
       </c>
       <c r="X24" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y24" t="b">
         <v>0</v>
@@ -2765,7 +2767,7 @@
         </is>
       </c>
       <c r="X25" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y25" t="b">
         <v>0</v>
@@ -2861,7 +2863,7 @@
         </is>
       </c>
       <c r="X26" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y26" t="b">
         <v>0</v>
@@ -2953,7 +2955,7 @@
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr"/>
       <c r="X27" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y27" t="b">
         <v>0</v>
@@ -3045,7 +3047,7 @@
       <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr"/>
       <c r="X28" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y28" t="b">
         <v>0</v>
@@ -3137,7 +3139,7 @@
       <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr"/>
       <c r="X29" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y29" t="b">
         <v>0</v>
@@ -3229,7 +3231,7 @@
       <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr"/>
       <c r="X30" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y30" t="b">
         <v>0</v>
@@ -3321,7 +3323,7 @@
       <c r="V31" t="inlineStr"/>
       <c r="W31" t="inlineStr"/>
       <c r="X31" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y31" t="b">
         <v>0</v>
@@ -3413,7 +3415,7 @@
       <c r="V32" t="inlineStr"/>
       <c r="W32" t="inlineStr"/>
       <c r="X32" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y32" t="b">
         <v>0</v>
@@ -3505,7 +3507,7 @@
       <c r="V33" t="inlineStr"/>
       <c r="W33" t="inlineStr"/>
       <c r="X33" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y33" t="b">
         <v>0</v>
@@ -3597,7 +3599,7 @@
       <c r="V34" t="inlineStr"/>
       <c r="W34" t="inlineStr"/>
       <c r="X34" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y34" t="b">
         <v>0</v>
@@ -3689,7 +3691,7 @@
       <c r="V35" t="inlineStr"/>
       <c r="W35" t="inlineStr"/>
       <c r="X35" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y35" t="b">
         <v>0</v>
@@ -3781,7 +3783,7 @@
       <c r="V36" t="inlineStr"/>
       <c r="W36" t="inlineStr"/>
       <c r="X36" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y36" t="b">
         <v>0</v>
@@ -3873,7 +3875,7 @@
       <c r="V37" t="inlineStr"/>
       <c r="W37" t="inlineStr"/>
       <c r="X37" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y37" t="b">
         <v>0</v>
@@ -3965,7 +3967,7 @@
       <c r="V38" t="inlineStr"/>
       <c r="W38" t="inlineStr"/>
       <c r="X38" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y38" t="b">
         <v>0</v>
@@ -4057,7 +4059,7 @@
       <c r="V39" t="inlineStr"/>
       <c r="W39" t="inlineStr"/>
       <c r="X39" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y39" t="b">
         <v>0</v>
@@ -4149,7 +4151,7 @@
       <c r="V40" t="inlineStr"/>
       <c r="W40" t="inlineStr"/>
       <c r="X40" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y40" t="b">
         <v>0</v>
@@ -4241,7 +4243,7 @@
       <c r="V41" t="inlineStr"/>
       <c r="W41" t="inlineStr"/>
       <c r="X41" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y41" t="b">
         <v>0</v>
@@ -4333,7 +4335,7 @@
       <c r="V42" t="inlineStr"/>
       <c r="W42" t="inlineStr"/>
       <c r="X42" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y42" t="b">
         <v>0</v>
@@ -4425,7 +4427,7 @@
       <c r="V43" t="inlineStr"/>
       <c r="W43" t="inlineStr"/>
       <c r="X43" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y43" t="b">
         <v>0</v>
@@ -4517,7 +4519,7 @@
       <c r="V44" t="inlineStr"/>
       <c r="W44" t="inlineStr"/>
       <c r="X44" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y44" t="b">
         <v>0</v>
@@ -4607,7 +4609,7 @@
         </is>
       </c>
       <c r="X45" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y45" t="b">
         <v>1</v>
@@ -4699,7 +4701,7 @@
       <c r="V46" t="inlineStr"/>
       <c r="W46" t="inlineStr"/>
       <c r="X46" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y46" t="b">
         <v>0</v>
@@ -4791,7 +4793,7 @@
       <c r="V47" t="inlineStr"/>
       <c r="W47" t="inlineStr"/>
       <c r="X47" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y47" t="b">
         <v>1</v>
@@ -4883,7 +4885,7 @@
       <c r="V48" t="inlineStr"/>
       <c r="W48" t="inlineStr"/>
       <c r="X48" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y48" t="b">
         <v>1</v>
@@ -4975,7 +4977,7 @@
       <c r="V49" t="inlineStr"/>
       <c r="W49" t="inlineStr"/>
       <c r="X49" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y49" t="b">
         <v>0</v>
@@ -5067,7 +5069,7 @@
       <c r="V50" t="inlineStr"/>
       <c r="W50" t="inlineStr"/>
       <c r="X50" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y50" t="b">
         <v>0</v>
@@ -5159,7 +5161,7 @@
       <c r="V51" t="inlineStr"/>
       <c r="W51" t="inlineStr"/>
       <c r="X51" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y51" t="b">
         <v>0</v>
@@ -5251,7 +5253,7 @@
       <c r="V52" t="inlineStr"/>
       <c r="W52" t="inlineStr"/>
       <c r="X52" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y52" t="b">
         <v>0</v>
@@ -5343,7 +5345,7 @@
       <c r="V53" t="inlineStr"/>
       <c r="W53" t="inlineStr"/>
       <c r="X53" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y53" t="b">
         <v>0</v>
@@ -5435,7 +5437,7 @@
       <c r="V54" t="inlineStr"/>
       <c r="W54" t="inlineStr"/>
       <c r="X54" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y54" t="b">
         <v>0</v>
@@ -5525,7 +5527,7 @@
       <c r="V55" t="inlineStr"/>
       <c r="W55" t="inlineStr"/>
       <c r="X55" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y55" t="b">
         <v>0</v>
@@ -5617,7 +5619,7 @@
       <c r="V56" t="inlineStr"/>
       <c r="W56" t="inlineStr"/>
       <c r="X56" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y56" t="b">
         <v>0</v>
@@ -5709,7 +5711,7 @@
       <c r="V57" t="inlineStr"/>
       <c r="W57" t="inlineStr"/>
       <c r="X57" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y57" t="b">
         <v>0</v>
@@ -5799,7 +5801,7 @@
       <c r="V58" t="inlineStr"/>
       <c r="W58" t="inlineStr"/>
       <c r="X58" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y58" t="b">
         <v>0</v>
@@ -5891,7 +5893,7 @@
       <c r="V59" t="inlineStr"/>
       <c r="W59" t="inlineStr"/>
       <c r="X59" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y59" t="b">
         <v>0</v>
@@ -5983,7 +5985,7 @@
       <c r="V60" t="inlineStr"/>
       <c r="W60" t="inlineStr"/>
       <c r="X60" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y60" t="b">
         <v>0</v>
@@ -6075,7 +6077,7 @@
       <c r="V61" t="inlineStr"/>
       <c r="W61" t="inlineStr"/>
       <c r="X61" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y61" t="b">
         <v>0</v>
@@ -6167,7 +6169,7 @@
       <c r="V62" t="inlineStr"/>
       <c r="W62" t="inlineStr"/>
       <c r="X62" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y62" t="b">
         <v>0</v>
@@ -6259,7 +6261,7 @@
       <c r="V63" t="inlineStr"/>
       <c r="W63" t="inlineStr"/>
       <c r="X63" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y63" t="b">
         <v>0</v>
@@ -6351,7 +6353,7 @@
       <c r="V64" t="inlineStr"/>
       <c r="W64" t="inlineStr"/>
       <c r="X64" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y64" t="b">
         <v>0</v>
@@ -6443,7 +6445,7 @@
       <c r="V65" t="inlineStr"/>
       <c r="W65" t="inlineStr"/>
       <c r="X65" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y65" t="b">
         <v>0</v>
@@ -6533,7 +6535,7 @@
       <c r="V66" t="inlineStr"/>
       <c r="W66" t="inlineStr"/>
       <c r="X66" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y66" t="b">
         <v>0</v>
@@ -6625,7 +6627,7 @@
       <c r="V67" t="inlineStr"/>
       <c r="W67" t="inlineStr"/>
       <c r="X67" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y67" t="b">
         <v>0</v>
@@ -6717,7 +6719,7 @@
       <c r="V68" t="inlineStr"/>
       <c r="W68" t="inlineStr"/>
       <c r="X68" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y68" t="b">
         <v>0</v>
@@ -6809,7 +6811,7 @@
       <c r="V69" t="inlineStr"/>
       <c r="W69" t="inlineStr"/>
       <c r="X69" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y69" t="b">
         <v>0</v>
@@ -6901,7 +6903,7 @@
       <c r="V70" t="inlineStr"/>
       <c r="W70" t="inlineStr"/>
       <c r="X70" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y70" t="b">
         <v>0</v>
@@ -6993,7 +6995,7 @@
       <c r="V71" t="inlineStr"/>
       <c r="W71" t="inlineStr"/>
       <c r="X71" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y71" t="b">
         <v>0</v>
@@ -7085,7 +7087,7 @@
       <c r="V72" t="inlineStr"/>
       <c r="W72" t="inlineStr"/>
       <c r="X72" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y72" t="b">
         <v>0</v>
@@ -7177,7 +7179,7 @@
       <c r="V73" t="inlineStr"/>
       <c r="W73" t="inlineStr"/>
       <c r="X73" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y73" t="b">
         <v>1</v>
@@ -7269,7 +7271,7 @@
       <c r="V74" t="inlineStr"/>
       <c r="W74" t="inlineStr"/>
       <c r="X74" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y74" t="b">
         <v>0</v>
@@ -7361,7 +7363,7 @@
       <c r="V75" t="inlineStr"/>
       <c r="W75" t="inlineStr"/>
       <c r="X75" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y75" t="b">
         <v>0</v>
@@ -7453,7 +7455,7 @@
       <c r="V76" t="inlineStr"/>
       <c r="W76" t="inlineStr"/>
       <c r="X76" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y76" t="b">
         <v>0</v>
@@ -7545,7 +7547,7 @@
       <c r="V77" t="inlineStr"/>
       <c r="W77" t="inlineStr"/>
       <c r="X77" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y77" t="b">
         <v>0</v>
@@ -7637,7 +7639,7 @@
       <c r="V78" t="inlineStr"/>
       <c r="W78" t="inlineStr"/>
       <c r="X78" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y78" t="b">
         <v>0</v>
@@ -7729,7 +7731,7 @@
       <c r="V79" t="inlineStr"/>
       <c r="W79" t="inlineStr"/>
       <c r="X79" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y79" t="b">
         <v>0</v>
@@ -7821,7 +7823,7 @@
       <c r="V80" t="inlineStr"/>
       <c r="W80" t="inlineStr"/>
       <c r="X80" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y80" t="b">
         <v>0</v>
@@ -7913,7 +7915,7 @@
       <c r="V81" t="inlineStr"/>
       <c r="W81" t="inlineStr"/>
       <c r="X81" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y81" t="b">
         <v>0</v>
@@ -8005,7 +8007,7 @@
       <c r="V82" t="inlineStr"/>
       <c r="W82" t="inlineStr"/>
       <c r="X82" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y82" t="b">
         <v>0</v>
@@ -8097,7 +8099,7 @@
       <c r="V83" t="inlineStr"/>
       <c r="W83" t="inlineStr"/>
       <c r="X83" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y83" t="b">
         <v>0</v>
@@ -8189,7 +8191,7 @@
       <c r="V84" t="inlineStr"/>
       <c r="W84" t="inlineStr"/>
       <c r="X84" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y84" t="b">
         <v>0</v>
@@ -8281,7 +8283,7 @@
       <c r="V85" t="inlineStr"/>
       <c r="W85" t="inlineStr"/>
       <c r="X85" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y85" t="b">
         <v>0</v>
@@ -8373,7 +8375,7 @@
       <c r="V86" t="inlineStr"/>
       <c r="W86" t="inlineStr"/>
       <c r="X86" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y86" t="b">
         <v>0</v>
@@ -8465,7 +8467,7 @@
       <c r="V87" t="inlineStr"/>
       <c r="W87" t="inlineStr"/>
       <c r="X87" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y87" t="b">
         <v>0</v>
@@ -8557,7 +8559,7 @@
       <c r="V88" t="inlineStr"/>
       <c r="W88" t="inlineStr"/>
       <c r="X88" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y88" t="b">
         <v>0</v>
@@ -8649,7 +8651,7 @@
       <c r="V89" t="inlineStr"/>
       <c r="W89" t="inlineStr"/>
       <c r="X89" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y89" t="b">
         <v>0</v>
@@ -8745,7 +8747,7 @@
       </c>
       <c r="W90" t="inlineStr"/>
       <c r="X90" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y90" t="b">
         <v>0</v>
@@ -8837,7 +8839,7 @@
       <c r="V91" t="inlineStr"/>
       <c r="W91" t="inlineStr"/>
       <c r="X91" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y91" t="b">
         <v>0</v>
@@ -8929,7 +8931,7 @@
       <c r="V92" t="inlineStr"/>
       <c r="W92" t="inlineStr"/>
       <c r="X92" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y92" t="b">
         <v>0</v>
@@ -9021,7 +9023,7 @@
       <c r="V93" t="inlineStr"/>
       <c r="W93" t="inlineStr"/>
       <c r="X93" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y93" t="b">
         <v>0</v>
@@ -9113,7 +9115,7 @@
       <c r="V94" t="inlineStr"/>
       <c r="W94" t="inlineStr"/>
       <c r="X94" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y94" t="b">
         <v>0</v>
@@ -9205,7 +9207,7 @@
       <c r="V95" t="inlineStr"/>
       <c r="W95" t="inlineStr"/>
       <c r="X95" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y95" t="b">
         <v>0</v>
@@ -9297,7 +9299,7 @@
       <c r="V96" t="inlineStr"/>
       <c r="W96" t="inlineStr"/>
       <c r="X96" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y96" t="b">
         <v>0</v>
@@ -9389,7 +9391,7 @@
       <c r="V97" t="inlineStr"/>
       <c r="W97" t="inlineStr"/>
       <c r="X97" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y97" t="b">
         <v>0</v>
@@ -9481,7 +9483,7 @@
       <c r="V98" t="inlineStr"/>
       <c r="W98" t="inlineStr"/>
       <c r="X98" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y98" t="b">
         <v>0</v>
@@ -9573,7 +9575,7 @@
       <c r="V99" t="inlineStr"/>
       <c r="W99" t="inlineStr"/>
       <c r="X99" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y99" t="b">
         <v>0</v>
@@ -9665,7 +9667,7 @@
       <c r="V100" t="inlineStr"/>
       <c r="W100" t="inlineStr"/>
       <c r="X100" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y100" t="b">
         <v>0</v>
@@ -9757,7 +9759,7 @@
       <c r="V101" t="inlineStr"/>
       <c r="W101" t="inlineStr"/>
       <c r="X101" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y101" t="b">
         <v>0</v>
@@ -9849,7 +9851,7 @@
       <c r="V102" t="inlineStr"/>
       <c r="W102" t="inlineStr"/>
       <c r="X102" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y102" t="b">
         <v>0</v>
@@ -9941,7 +9943,7 @@
       <c r="V103" t="inlineStr"/>
       <c r="W103" t="inlineStr"/>
       <c r="X103" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y103" t="b">
         <v>0</v>
@@ -10033,7 +10035,7 @@
       <c r="V104" t="inlineStr"/>
       <c r="W104" t="inlineStr"/>
       <c r="X104" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y104" t="b">
         <v>0</v>
@@ -10125,7 +10127,7 @@
       <c r="V105" t="inlineStr"/>
       <c r="W105" t="inlineStr"/>
       <c r="X105" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y105" t="b">
         <v>0</v>
@@ -10217,7 +10219,7 @@
       <c r="V106" t="inlineStr"/>
       <c r="W106" t="inlineStr"/>
       <c r="X106" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y106" t="b">
         <v>0</v>
@@ -10309,7 +10311,7 @@
       <c r="V107" t="inlineStr"/>
       <c r="W107" t="inlineStr"/>
       <c r="X107" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y107" t="b">
         <v>0</v>
@@ -10401,7 +10403,7 @@
       <c r="V108" t="inlineStr"/>
       <c r="W108" t="inlineStr"/>
       <c r="X108" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y108" t="b">
         <v>0</v>
@@ -10493,7 +10495,7 @@
       <c r="V109" t="inlineStr"/>
       <c r="W109" t="inlineStr"/>
       <c r="X109" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y109" t="b">
         <v>0</v>
@@ -10585,7 +10587,7 @@
         </is>
       </c>
       <c r="X110" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y110" t="b">
         <v>1</v>
@@ -10677,7 +10679,7 @@
         </is>
       </c>
       <c r="X111" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y111" t="b">
         <v>1</v>
@@ -10769,7 +10771,7 @@
       <c r="V112" t="inlineStr"/>
       <c r="W112" t="inlineStr"/>
       <c r="X112" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y112" t="b">
         <v>1</v>
@@ -10861,7 +10863,7 @@
         </is>
       </c>
       <c r="X113" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y113" t="b">
         <v>1</v>
@@ -10957,7 +10959,7 @@
         </is>
       </c>
       <c r="X114" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y114" t="b">
         <v>0</v>
@@ -11049,7 +11051,7 @@
       <c r="V115" t="inlineStr"/>
       <c r="W115" t="inlineStr"/>
       <c r="X115" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y115" t="b">
         <v>0</v>
@@ -11145,7 +11147,7 @@
         </is>
       </c>
       <c r="X116" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y116" t="b">
         <v>0</v>
@@ -11237,7 +11239,7 @@
       <c r="V117" t="inlineStr"/>
       <c r="W117" t="inlineStr"/>
       <c r="X117" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y117" t="b">
         <v>0</v>
@@ -11327,7 +11329,7 @@
         </is>
       </c>
       <c r="X118" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y118" t="b">
         <v>1</v>
@@ -11417,7 +11419,7 @@
         </is>
       </c>
       <c r="X119" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y119" t="b">
         <v>1</v>
@@ -11507,7 +11509,7 @@
         </is>
       </c>
       <c r="X120" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y120" t="b">
         <v>1</v>
@@ -11599,7 +11601,7 @@
       <c r="V121" t="inlineStr"/>
       <c r="W121" t="inlineStr"/>
       <c r="X121" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y121" t="b">
         <v>0</v>
@@ -11691,7 +11693,7 @@
       <c r="V122" t="inlineStr"/>
       <c r="W122" t="inlineStr"/>
       <c r="X122" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y122" t="b">
         <v>0</v>
@@ -11783,7 +11785,7 @@
       <c r="V123" t="inlineStr"/>
       <c r="W123" t="inlineStr"/>
       <c r="X123" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y123" t="b">
         <v>0</v>
@@ -11875,7 +11877,7 @@
       <c r="V124" t="inlineStr"/>
       <c r="W124" t="inlineStr"/>
       <c r="X124" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y124" t="b">
         <v>1</v>
@@ -11967,7 +11969,7 @@
       <c r="V125" t="inlineStr"/>
       <c r="W125" t="inlineStr"/>
       <c r="X125" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y125" t="b">
         <v>0</v>
@@ -12059,7 +12061,7 @@
       <c r="V126" t="inlineStr"/>
       <c r="W126" t="inlineStr"/>
       <c r="X126" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y126" t="b">
         <v>0</v>
@@ -12151,7 +12153,7 @@
       <c r="V127" t="inlineStr"/>
       <c r="W127" t="inlineStr"/>
       <c r="X127" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y127" t="b">
         <v>0</v>
@@ -12243,7 +12245,7 @@
       <c r="V128" t="inlineStr"/>
       <c r="W128" t="inlineStr"/>
       <c r="X128" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y128" t="b">
         <v>0</v>
@@ -12335,7 +12337,7 @@
       <c r="V129" t="inlineStr"/>
       <c r="W129" t="inlineStr"/>
       <c r="X129" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y129" t="b">
         <v>0</v>
@@ -12427,7 +12429,7 @@
       <c r="V130" t="inlineStr"/>
       <c r="W130" t="inlineStr"/>
       <c r="X130" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y130" t="b">
         <v>0</v>
@@ -12519,7 +12521,7 @@
       <c r="V131" t="inlineStr"/>
       <c r="W131" t="inlineStr"/>
       <c r="X131" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y131" t="b">
         <v>0</v>
@@ -12611,7 +12613,7 @@
       <c r="V132" t="inlineStr"/>
       <c r="W132" t="inlineStr"/>
       <c r="X132" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y132" t="b">
         <v>0</v>
@@ -12703,7 +12705,7 @@
       <c r="V133" t="inlineStr"/>
       <c r="W133" t="inlineStr"/>
       <c r="X133" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y133" t="b">
         <v>0</v>
@@ -12795,7 +12797,7 @@
       <c r="V134" t="inlineStr"/>
       <c r="W134" t="inlineStr"/>
       <c r="X134" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y134" t="b">
         <v>0</v>
@@ -12887,7 +12889,7 @@
       <c r="V135" t="inlineStr"/>
       <c r="W135" t="inlineStr"/>
       <c r="X135" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y135" t="b">
         <v>0</v>
@@ -12979,7 +12981,7 @@
       <c r="V136" t="inlineStr"/>
       <c r="W136" t="inlineStr"/>
       <c r="X136" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y136" t="b">
         <v>0</v>
@@ -13071,7 +13073,7 @@
       <c r="V137" t="inlineStr"/>
       <c r="W137" t="inlineStr"/>
       <c r="X137" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y137" t="b">
         <v>0</v>
@@ -13163,7 +13165,7 @@
       <c r="V138" t="inlineStr"/>
       <c r="W138" t="inlineStr"/>
       <c r="X138" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y138" t="b">
         <v>0</v>
@@ -13255,7 +13257,7 @@
       <c r="V139" t="inlineStr"/>
       <c r="W139" t="inlineStr"/>
       <c r="X139" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y139" t="b">
         <v>0</v>
@@ -13345,7 +13347,7 @@
       <c r="V140" t="inlineStr"/>
       <c r="W140" t="inlineStr"/>
       <c r="X140" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y140" t="b">
         <v>0</v>
@@ -13437,7 +13439,7 @@
       <c r="V141" t="inlineStr"/>
       <c r="W141" t="inlineStr"/>
       <c r="X141" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y141" t="b">
         <v>0</v>
@@ -13529,7 +13531,7 @@
       <c r="V142" t="inlineStr"/>
       <c r="W142" t="inlineStr"/>
       <c r="X142" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y142" t="b">
         <v>0</v>
@@ -13621,7 +13623,7 @@
       <c r="V143" t="inlineStr"/>
       <c r="W143" t="inlineStr"/>
       <c r="X143" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y143" t="b">
         <v>0</v>
@@ -13713,7 +13715,7 @@
       <c r="V144" t="inlineStr"/>
       <c r="W144" t="inlineStr"/>
       <c r="X144" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y144" t="b">
         <v>0</v>
@@ -13805,7 +13807,7 @@
       <c r="V145" t="inlineStr"/>
       <c r="W145" t="inlineStr"/>
       <c r="X145" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y145" t="b">
         <v>0</v>
@@ -13897,7 +13899,7 @@
       <c r="V146" t="inlineStr"/>
       <c r="W146" t="inlineStr"/>
       <c r="X146" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y146" t="b">
         <v>0</v>
@@ -13989,7 +13991,7 @@
       <c r="V147" t="inlineStr"/>
       <c r="W147" t="inlineStr"/>
       <c r="X147" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y147" t="b">
         <v>0</v>
@@ -14081,7 +14083,7 @@
       <c r="V148" t="inlineStr"/>
       <c r="W148" t="inlineStr"/>
       <c r="X148" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y148" t="b">
         <v>0</v>
@@ -14173,7 +14175,7 @@
       <c r="V149" t="inlineStr"/>
       <c r="W149" t="inlineStr"/>
       <c r="X149" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y149" t="b">
         <v>0</v>
@@ -14265,7 +14267,7 @@
       <c r="V150" t="inlineStr"/>
       <c r="W150" t="inlineStr"/>
       <c r="X150" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y150" t="b">
         <v>0</v>
@@ -14357,7 +14359,7 @@
       <c r="V151" t="inlineStr"/>
       <c r="W151" t="inlineStr"/>
       <c r="X151" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y151" t="b">
         <v>0</v>
@@ -14449,7 +14451,7 @@
       <c r="V152" t="inlineStr"/>
       <c r="W152" t="inlineStr"/>
       <c r="X152" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y152" t="b">
         <v>0</v>
@@ -14541,7 +14543,7 @@
       <c r="V153" t="inlineStr"/>
       <c r="W153" t="inlineStr"/>
       <c r="X153" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y153" t="b">
         <v>0</v>
@@ -14633,7 +14635,7 @@
       <c r="V154" t="inlineStr"/>
       <c r="W154" t="inlineStr"/>
       <c r="X154" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y154" t="b">
         <v>0</v>
@@ -14725,7 +14727,7 @@
       <c r="V155" t="inlineStr"/>
       <c r="W155" t="inlineStr"/>
       <c r="X155" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y155" t="b">
         <v>0</v>
@@ -14817,7 +14819,7 @@
       <c r="V156" t="inlineStr"/>
       <c r="W156" t="inlineStr"/>
       <c r="X156" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y156" t="b">
         <v>0</v>
@@ -14909,7 +14911,7 @@
       <c r="V157" t="inlineStr"/>
       <c r="W157" t="inlineStr"/>
       <c r="X157" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y157" t="b">
         <v>0</v>
@@ -15001,7 +15003,7 @@
       <c r="V158" t="inlineStr"/>
       <c r="W158" t="inlineStr"/>
       <c r="X158" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y158" t="b">
         <v>0</v>
@@ -15093,7 +15095,7 @@
       <c r="V159" t="inlineStr"/>
       <c r="W159" t="inlineStr"/>
       <c r="X159" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y159" t="b">
         <v>0</v>
@@ -15181,7 +15183,7 @@
         </is>
       </c>
       <c r="X160" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y160" t="b">
         <v>1</v>
@@ -15273,7 +15275,7 @@
       <c r="V161" t="inlineStr"/>
       <c r="W161" t="inlineStr"/>
       <c r="X161" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y161" t="b">
         <v>0</v>
@@ -15365,7 +15367,7 @@
       <c r="V162" t="inlineStr"/>
       <c r="W162" t="inlineStr"/>
       <c r="X162" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y162" t="b">
         <v>0</v>
@@ -15457,7 +15459,7 @@
       <c r="V163" t="inlineStr"/>
       <c r="W163" t="inlineStr"/>
       <c r="X163" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y163" t="b">
         <v>0</v>
@@ -15549,7 +15551,7 @@
       <c r="V164" t="inlineStr"/>
       <c r="W164" t="inlineStr"/>
       <c r="X164" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y164" t="b">
         <v>0</v>
@@ -15641,7 +15643,7 @@
       <c r="V165" t="inlineStr"/>
       <c r="W165" t="inlineStr"/>
       <c r="X165" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y165" t="b">
         <v>0</v>
@@ -15733,7 +15735,7 @@
       <c r="V166" t="inlineStr"/>
       <c r="W166" t="inlineStr"/>
       <c r="X166" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y166" t="b">
         <v>0</v>
@@ -15825,7 +15827,7 @@
       <c r="V167" t="inlineStr"/>
       <c r="W167" t="inlineStr"/>
       <c r="X167" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y167" t="b">
         <v>0</v>
@@ -15917,7 +15919,7 @@
       <c r="V168" t="inlineStr"/>
       <c r="W168" t="inlineStr"/>
       <c r="X168" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y168" t="b">
         <v>0</v>
@@ -16009,7 +16011,7 @@
       <c r="V169" t="inlineStr"/>
       <c r="W169" t="inlineStr"/>
       <c r="X169" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y169" t="b">
         <v>0</v>
@@ -16101,7 +16103,7 @@
       <c r="V170" t="inlineStr"/>
       <c r="W170" t="inlineStr"/>
       <c r="X170" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y170" t="b">
         <v>0</v>
@@ -16193,7 +16195,7 @@
       <c r="V171" t="inlineStr"/>
       <c r="W171" t="inlineStr"/>
       <c r="X171" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y171" t="b">
         <v>0</v>
@@ -16285,7 +16287,7 @@
       <c r="V172" t="inlineStr"/>
       <c r="W172" t="inlineStr"/>
       <c r="X172" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y172" t="b">
         <v>0</v>
@@ -16377,7 +16379,7 @@
       <c r="V173" t="inlineStr"/>
       <c r="W173" t="inlineStr"/>
       <c r="X173" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y173" t="b">
         <v>1</v>
@@ -16469,7 +16471,7 @@
       <c r="V174" t="inlineStr"/>
       <c r="W174" t="inlineStr"/>
       <c r="X174" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y174" t="b">
         <v>0</v>
@@ -16561,7 +16563,7 @@
       <c r="V175" t="inlineStr"/>
       <c r="W175" t="inlineStr"/>
       <c r="X175" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y175" t="b">
         <v>0</v>
@@ -16653,7 +16655,7 @@
       <c r="V176" t="inlineStr"/>
       <c r="W176" t="inlineStr"/>
       <c r="X176" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y176" t="b">
         <v>0</v>
@@ -16745,7 +16747,7 @@
       <c r="V177" t="inlineStr"/>
       <c r="W177" t="inlineStr"/>
       <c r="X177" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y177" t="b">
         <v>0</v>
@@ -16837,7 +16839,7 @@
       <c r="V178" t="inlineStr"/>
       <c r="W178" t="inlineStr"/>
       <c r="X178" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y178" t="b">
         <v>0</v>
@@ -16929,7 +16931,7 @@
       <c r="V179" t="inlineStr"/>
       <c r="W179" t="inlineStr"/>
       <c r="X179" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y179" t="b">
         <v>0</v>
@@ -17021,7 +17023,7 @@
       <c r="V180" t="inlineStr"/>
       <c r="W180" t="inlineStr"/>
       <c r="X180" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y180" t="b">
         <v>0</v>
@@ -17113,7 +17115,7 @@
       <c r="V181" t="inlineStr"/>
       <c r="W181" t="inlineStr"/>
       <c r="X181" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y181" t="b">
         <v>0</v>
@@ -17205,7 +17207,7 @@
       <c r="V182" t="inlineStr"/>
       <c r="W182" t="inlineStr"/>
       <c r="X182" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y182" t="b">
         <v>0</v>
@@ -17297,7 +17299,7 @@
       <c r="V183" t="inlineStr"/>
       <c r="W183" t="inlineStr"/>
       <c r="X183" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y183" t="b">
         <v>0</v>
@@ -17389,7 +17391,7 @@
         </is>
       </c>
       <c r="X184" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y184" t="b">
         <v>0</v>
@@ -17481,7 +17483,7 @@
       <c r="V185" t="inlineStr"/>
       <c r="W185" t="inlineStr"/>
       <c r="X185" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y185" t="b">
         <v>0</v>
@@ -17573,7 +17575,7 @@
       <c r="V186" t="inlineStr"/>
       <c r="W186" t="inlineStr"/>
       <c r="X186" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y186" t="b">
         <v>0</v>
@@ -17665,7 +17667,7 @@
       <c r="V187" t="inlineStr"/>
       <c r="W187" t="inlineStr"/>
       <c r="X187" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y187" t="b">
         <v>0</v>
@@ -17757,7 +17759,7 @@
       <c r="V188" t="inlineStr"/>
       <c r="W188" t="inlineStr"/>
       <c r="X188" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y188" t="b">
         <v>0</v>
@@ -17855,7 +17857,7 @@
         </is>
       </c>
       <c r="X189" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y189" t="b">
         <v>0</v>
@@ -17953,7 +17955,7 @@
         </is>
       </c>
       <c r="X190" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y190" t="b">
         <v>0</v>
@@ -18045,7 +18047,7 @@
       <c r="V191" t="inlineStr"/>
       <c r="W191" t="inlineStr"/>
       <c r="X191" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y191" t="b">
         <v>0</v>
@@ -18137,7 +18139,7 @@
       <c r="V192" t="inlineStr"/>
       <c r="W192" t="inlineStr"/>
       <c r="X192" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y192" t="b">
         <v>0</v>
@@ -18229,7 +18231,7 @@
       <c r="V193" t="inlineStr"/>
       <c r="W193" t="inlineStr"/>
       <c r="X193" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y193" t="b">
         <v>0</v>
@@ -18321,7 +18323,7 @@
       <c r="V194" t="inlineStr"/>
       <c r="W194" t="inlineStr"/>
       <c r="X194" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y194" t="b">
         <v>0</v>
@@ -18419,7 +18421,7 @@
         </is>
       </c>
       <c r="X195" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y195" t="b">
         <v>0</v>
@@ -18511,7 +18513,7 @@
       <c r="V196" t="inlineStr"/>
       <c r="W196" t="inlineStr"/>
       <c r="X196" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y196" t="b">
         <v>0</v>
@@ -18603,7 +18605,7 @@
       <c r="V197" t="inlineStr"/>
       <c r="W197" t="inlineStr"/>
       <c r="X197" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y197" t="b">
         <v>0</v>
@@ -18701,7 +18703,7 @@
         </is>
       </c>
       <c r="X198" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y198" t="b">
         <v>0</v>
@@ -18793,7 +18795,7 @@
       <c r="V199" t="inlineStr"/>
       <c r="W199" t="inlineStr"/>
       <c r="X199" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y199" t="b">
         <v>0</v>
@@ -18885,7 +18887,7 @@
       <c r="V200" t="inlineStr"/>
       <c r="W200" t="inlineStr"/>
       <c r="X200" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y200" t="b">
         <v>0</v>
@@ -18983,7 +18985,7 @@
         </is>
       </c>
       <c r="X201" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y201" t="b">
         <v>0</v>
@@ -19081,7 +19083,7 @@
         </is>
       </c>
       <c r="X202" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y202" t="b">
         <v>0</v>
@@ -19173,7 +19175,7 @@
       <c r="V203" t="inlineStr"/>
       <c r="W203" t="inlineStr"/>
       <c r="X203" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y203" t="b">
         <v>0</v>
@@ -19265,7 +19267,7 @@
       <c r="V204" t="inlineStr"/>
       <c r="W204" t="inlineStr"/>
       <c r="X204" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y204" t="b">
         <v>0</v>
@@ -19357,7 +19359,7 @@
       <c r="V205" t="inlineStr"/>
       <c r="W205" t="inlineStr"/>
       <c r="X205" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y205" t="b">
         <v>0</v>
@@ -19449,7 +19451,7 @@
       <c r="V206" t="inlineStr"/>
       <c r="W206" t="inlineStr"/>
       <c r="X206" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y206" t="b">
         <v>0</v>
@@ -19541,7 +19543,7 @@
       <c r="V207" t="inlineStr"/>
       <c r="W207" t="inlineStr"/>
       <c r="X207" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y207" t="b">
         <v>0</v>
@@ -19633,7 +19635,7 @@
       <c r="V208" t="inlineStr"/>
       <c r="W208" t="inlineStr"/>
       <c r="X208" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y208" t="b">
         <v>0</v>
@@ -19725,7 +19727,7 @@
       <c r="V209" t="inlineStr"/>
       <c r="W209" t="inlineStr"/>
       <c r="X209" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y209" t="b">
         <v>1</v>
@@ -19817,7 +19819,7 @@
       <c r="V210" t="inlineStr"/>
       <c r="W210" t="inlineStr"/>
       <c r="X210" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y210" t="b">
         <v>1</v>
@@ -19909,7 +19911,7 @@
       <c r="V211" t="inlineStr"/>
       <c r="W211" t="inlineStr"/>
       <c r="X211" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y211" t="b">
         <v>1</v>
@@ -20001,7 +20003,7 @@
       <c r="V212" t="inlineStr"/>
       <c r="W212" t="inlineStr"/>
       <c r="X212" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y212" t="b">
         <v>0</v>
@@ -20093,7 +20095,7 @@
       <c r="V213" t="inlineStr"/>
       <c r="W213" t="inlineStr"/>
       <c r="X213" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y213" t="b">
         <v>0</v>
@@ -20185,7 +20187,7 @@
       <c r="V214" t="inlineStr"/>
       <c r="W214" t="inlineStr"/>
       <c r="X214" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y214" t="b">
         <v>0</v>
@@ -20277,7 +20279,7 @@
       <c r="V215" t="inlineStr"/>
       <c r="W215" t="inlineStr"/>
       <c r="X215" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y215" t="b">
         <v>0</v>
@@ -20369,7 +20371,7 @@
       <c r="V216" t="inlineStr"/>
       <c r="W216" t="inlineStr"/>
       <c r="X216" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y216" t="b">
         <v>0</v>
@@ -20461,7 +20463,7 @@
       <c r="V217" t="inlineStr"/>
       <c r="W217" t="inlineStr"/>
       <c r="X217" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y217" t="b">
         <v>0</v>
@@ -20553,7 +20555,7 @@
       <c r="V218" t="inlineStr"/>
       <c r="W218" t="inlineStr"/>
       <c r="X218" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y218" t="b">
         <v>0</v>
@@ -20645,7 +20647,7 @@
       <c r="V219" t="inlineStr"/>
       <c r="W219" t="inlineStr"/>
       <c r="X219" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y219" t="b">
         <v>0</v>
@@ -20741,7 +20743,7 @@
         </is>
       </c>
       <c r="X220" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y220" t="b">
         <v>0</v>
@@ -20833,7 +20835,7 @@
       <c r="V221" t="inlineStr"/>
       <c r="W221" t="inlineStr"/>
       <c r="X221" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y221" t="b">
         <v>0</v>
@@ -20925,7 +20927,7 @@
       <c r="V222" t="inlineStr"/>
       <c r="W222" t="inlineStr"/>
       <c r="X222" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y222" t="b">
         <v>0</v>
@@ -21017,7 +21019,7 @@
       <c r="V223" t="inlineStr"/>
       <c r="W223" t="inlineStr"/>
       <c r="X223" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y223" t="b">
         <v>0</v>
@@ -21113,7 +21115,7 @@
         </is>
       </c>
       <c r="X224" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y224" t="b">
         <v>0</v>
@@ -21205,7 +21207,7 @@
       <c r="V225" t="inlineStr"/>
       <c r="W225" t="inlineStr"/>
       <c r="X225" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y225" t="b">
         <v>0</v>
@@ -21297,7 +21299,7 @@
       <c r="V226" t="inlineStr"/>
       <c r="W226" t="inlineStr"/>
       <c r="X226" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y226" t="b">
         <v>0</v>
@@ -21389,7 +21391,7 @@
       <c r="V227" t="inlineStr"/>
       <c r="W227" t="inlineStr"/>
       <c r="X227" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y227" t="b">
         <v>0</v>
@@ -21481,7 +21483,7 @@
       <c r="V228" t="inlineStr"/>
       <c r="W228" t="inlineStr"/>
       <c r="X228" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y228" t="b">
         <v>0</v>
@@ -21569,7 +21571,7 @@
       </c>
       <c r="W229" t="inlineStr"/>
       <c r="X229" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y229" t="b">
         <v>1</v>
@@ -21657,7 +21659,7 @@
       <c r="V230" t="inlineStr"/>
       <c r="W230" t="inlineStr"/>
       <c r="X230" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y230" t="b">
         <v>0</v>
@@ -21753,7 +21755,7 @@
       </c>
       <c r="W231" t="inlineStr"/>
       <c r="X231" s="2" t="n">
-        <v>46290.49412037037</v>
+        <v>46290.83268518518</v>
       </c>
       <c r="Y231" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Update data package at: 2026-09-28T07:58:33Z
</commit_message>
<xml_diff>
--- a/data/dados_sigplan_2027/indicadores_planejamento.xlsx
+++ b/data/dados_sigplan_2027/indicadores_planejamento.xlsx
@@ -645,7 +645,7 @@
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
       <c r="X2" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y2" t="b">
         <v>0</v>
@@ -737,7 +737,7 @@
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
       <c r="X3" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y3" t="b">
         <v>0</v>
@@ -829,7 +829,7 @@
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
       <c r="X4" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y4" t="b">
         <v>1</v>
@@ -921,7 +921,7 @@
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr"/>
       <c r="X5" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y5" t="b">
         <v>1</v>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="W6" t="inlineStr"/>
       <c r="X6" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y6" t="b">
         <v>0</v>
@@ -1109,7 +1109,7 @@
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
       <c r="X7" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y7" t="b">
         <v>0</v>
@@ -1201,7 +1201,7 @@
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
       <c r="X8" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y8" t="b">
         <v>0</v>
@@ -1293,7 +1293,7 @@
         </is>
       </c>
       <c r="X9" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y9" t="b">
         <v>0</v>
@@ -1385,7 +1385,7 @@
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
       <c r="X10" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y10" t="b">
         <v>0</v>
@@ -1477,7 +1477,7 @@
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
       <c r="X11" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y11" t="b">
         <v>0</v>
@@ -1569,7 +1569,7 @@
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
       <c r="X12" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y12" t="b">
         <v>0</v>
@@ -1661,7 +1661,7 @@
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr"/>
       <c r="X13" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y13" t="b">
         <v>0</v>
@@ -1753,7 +1753,7 @@
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
       <c r="X14" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y14" t="b">
         <v>0</v>
@@ -1845,7 +1845,7 @@
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
       <c r="X15" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y15" t="b">
         <v>1</v>
@@ -1937,7 +1937,7 @@
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
       <c r="X16" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y16" t="b">
         <v>0</v>
@@ -2029,7 +2029,7 @@
       <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
       <c r="X17" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y17" t="b">
         <v>0</v>
@@ -2121,7 +2121,7 @@
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr"/>
       <c r="X18" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y18" t="b">
         <v>0</v>
@@ -2213,7 +2213,7 @@
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
       <c r="X19" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y19" t="b">
         <v>0</v>
@@ -2305,7 +2305,7 @@
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr"/>
       <c r="X20" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y20" t="b">
         <v>0</v>
@@ -2397,7 +2397,7 @@
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
       <c r="X21" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y21" t="b">
         <v>0</v>
@@ -2489,7 +2489,7 @@
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr"/>
       <c r="X22" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y22" t="b">
         <v>0</v>
@@ -2581,7 +2581,7 @@
       <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr"/>
       <c r="X23" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y23" t="b">
         <v>0</v>
@@ -2671,7 +2671,7 @@
         </is>
       </c>
       <c r="X24" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y24" t="b">
         <v>0</v>
@@ -2767,7 +2767,7 @@
         </is>
       </c>
       <c r="X25" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y25" t="b">
         <v>0</v>
@@ -2863,7 +2863,7 @@
         </is>
       </c>
       <c r="X26" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y26" t="b">
         <v>0</v>
@@ -2955,7 +2955,7 @@
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr"/>
       <c r="X27" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y27" t="b">
         <v>0</v>
@@ -3047,7 +3047,7 @@
       <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr"/>
       <c r="X28" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y28" t="b">
         <v>0</v>
@@ -3139,7 +3139,7 @@
       <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr"/>
       <c r="X29" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y29" t="b">
         <v>0</v>
@@ -3231,7 +3231,7 @@
       <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr"/>
       <c r="X30" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y30" t="b">
         <v>0</v>
@@ -3323,7 +3323,7 @@
       <c r="V31" t="inlineStr"/>
       <c r="W31" t="inlineStr"/>
       <c r="X31" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y31" t="b">
         <v>0</v>
@@ -3415,7 +3415,7 @@
       <c r="V32" t="inlineStr"/>
       <c r="W32" t="inlineStr"/>
       <c r="X32" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y32" t="b">
         <v>0</v>
@@ -3507,7 +3507,7 @@
       <c r="V33" t="inlineStr"/>
       <c r="W33" t="inlineStr"/>
       <c r="X33" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y33" t="b">
         <v>0</v>
@@ -3599,7 +3599,7 @@
       <c r="V34" t="inlineStr"/>
       <c r="W34" t="inlineStr"/>
       <c r="X34" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y34" t="b">
         <v>0</v>
@@ -3691,7 +3691,7 @@
       <c r="V35" t="inlineStr"/>
       <c r="W35" t="inlineStr"/>
       <c r="X35" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y35" t="b">
         <v>0</v>
@@ -3783,7 +3783,7 @@
       <c r="V36" t="inlineStr"/>
       <c r="W36" t="inlineStr"/>
       <c r="X36" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y36" t="b">
         <v>0</v>
@@ -3875,7 +3875,7 @@
       <c r="V37" t="inlineStr"/>
       <c r="W37" t="inlineStr"/>
       <c r="X37" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y37" t="b">
         <v>0</v>
@@ -3967,7 +3967,7 @@
       <c r="V38" t="inlineStr"/>
       <c r="W38" t="inlineStr"/>
       <c r="X38" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y38" t="b">
         <v>0</v>
@@ -4059,7 +4059,7 @@
       <c r="V39" t="inlineStr"/>
       <c r="W39" t="inlineStr"/>
       <c r="X39" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y39" t="b">
         <v>0</v>
@@ -4151,7 +4151,7 @@
       <c r="V40" t="inlineStr"/>
       <c r="W40" t="inlineStr"/>
       <c r="X40" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y40" t="b">
         <v>0</v>
@@ -4243,7 +4243,7 @@
       <c r="V41" t="inlineStr"/>
       <c r="W41" t="inlineStr"/>
       <c r="X41" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y41" t="b">
         <v>0</v>
@@ -4335,7 +4335,7 @@
       <c r="V42" t="inlineStr"/>
       <c r="W42" t="inlineStr"/>
       <c r="X42" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y42" t="b">
         <v>0</v>
@@ -4427,7 +4427,7 @@
       <c r="V43" t="inlineStr"/>
       <c r="W43" t="inlineStr"/>
       <c r="X43" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y43" t="b">
         <v>0</v>
@@ -4519,7 +4519,7 @@
       <c r="V44" t="inlineStr"/>
       <c r="W44" t="inlineStr"/>
       <c r="X44" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y44" t="b">
         <v>0</v>
@@ -4609,7 +4609,7 @@
         </is>
       </c>
       <c r="X45" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y45" t="b">
         <v>1</v>
@@ -4701,7 +4701,7 @@
       <c r="V46" t="inlineStr"/>
       <c r="W46" t="inlineStr"/>
       <c r="X46" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y46" t="b">
         <v>0</v>
@@ -4793,7 +4793,7 @@
       <c r="V47" t="inlineStr"/>
       <c r="W47" t="inlineStr"/>
       <c r="X47" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y47" t="b">
         <v>1</v>
@@ -4885,7 +4885,7 @@
       <c r="V48" t="inlineStr"/>
       <c r="W48" t="inlineStr"/>
       <c r="X48" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y48" t="b">
         <v>1</v>
@@ -4977,7 +4977,7 @@
       <c r="V49" t="inlineStr"/>
       <c r="W49" t="inlineStr"/>
       <c r="X49" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y49" t="b">
         <v>0</v>
@@ -5069,7 +5069,7 @@
       <c r="V50" t="inlineStr"/>
       <c r="W50" t="inlineStr"/>
       <c r="X50" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y50" t="b">
         <v>0</v>
@@ -5161,7 +5161,7 @@
       <c r="V51" t="inlineStr"/>
       <c r="W51" t="inlineStr"/>
       <c r="X51" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y51" t="b">
         <v>0</v>
@@ -5253,7 +5253,7 @@
       <c r="V52" t="inlineStr"/>
       <c r="W52" t="inlineStr"/>
       <c r="X52" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y52" t="b">
         <v>0</v>
@@ -5345,7 +5345,7 @@
       <c r="V53" t="inlineStr"/>
       <c r="W53" t="inlineStr"/>
       <c r="X53" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y53" t="b">
         <v>0</v>
@@ -5437,7 +5437,7 @@
       <c r="V54" t="inlineStr"/>
       <c r="W54" t="inlineStr"/>
       <c r="X54" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y54" t="b">
         <v>0</v>
@@ -5527,7 +5527,7 @@
       <c r="V55" t="inlineStr"/>
       <c r="W55" t="inlineStr"/>
       <c r="X55" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y55" t="b">
         <v>0</v>
@@ -5619,7 +5619,7 @@
       <c r="V56" t="inlineStr"/>
       <c r="W56" t="inlineStr"/>
       <c r="X56" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y56" t="b">
         <v>0</v>
@@ -5711,7 +5711,7 @@
       <c r="V57" t="inlineStr"/>
       <c r="W57" t="inlineStr"/>
       <c r="X57" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y57" t="b">
         <v>0</v>
@@ -5801,7 +5801,7 @@
       <c r="V58" t="inlineStr"/>
       <c r="W58" t="inlineStr"/>
       <c r="X58" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y58" t="b">
         <v>0</v>
@@ -5893,7 +5893,7 @@
       <c r="V59" t="inlineStr"/>
       <c r="W59" t="inlineStr"/>
       <c r="X59" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y59" t="b">
         <v>0</v>
@@ -5985,7 +5985,7 @@
       <c r="V60" t="inlineStr"/>
       <c r="W60" t="inlineStr"/>
       <c r="X60" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y60" t="b">
         <v>0</v>
@@ -6077,7 +6077,7 @@
       <c r="V61" t="inlineStr"/>
       <c r="W61" t="inlineStr"/>
       <c r="X61" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y61" t="b">
         <v>0</v>
@@ -6169,7 +6169,7 @@
       <c r="V62" t="inlineStr"/>
       <c r="W62" t="inlineStr"/>
       <c r="X62" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y62" t="b">
         <v>0</v>
@@ -6261,7 +6261,7 @@
       <c r="V63" t="inlineStr"/>
       <c r="W63" t="inlineStr"/>
       <c r="X63" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y63" t="b">
         <v>0</v>
@@ -6353,7 +6353,7 @@
       <c r="V64" t="inlineStr"/>
       <c r="W64" t="inlineStr"/>
       <c r="X64" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y64" t="b">
         <v>0</v>
@@ -6445,7 +6445,7 @@
       <c r="V65" t="inlineStr"/>
       <c r="W65" t="inlineStr"/>
       <c r="X65" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y65" t="b">
         <v>0</v>
@@ -6535,7 +6535,7 @@
       <c r="V66" t="inlineStr"/>
       <c r="W66" t="inlineStr"/>
       <c r="X66" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y66" t="b">
         <v>0</v>
@@ -6627,7 +6627,7 @@
       <c r="V67" t="inlineStr"/>
       <c r="W67" t="inlineStr"/>
       <c r="X67" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y67" t="b">
         <v>0</v>
@@ -6719,7 +6719,7 @@
       <c r="V68" t="inlineStr"/>
       <c r="W68" t="inlineStr"/>
       <c r="X68" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y68" t="b">
         <v>0</v>
@@ -6811,7 +6811,7 @@
       <c r="V69" t="inlineStr"/>
       <c r="W69" t="inlineStr"/>
       <c r="X69" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y69" t="b">
         <v>0</v>
@@ -6903,7 +6903,7 @@
       <c r="V70" t="inlineStr"/>
       <c r="W70" t="inlineStr"/>
       <c r="X70" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y70" t="b">
         <v>0</v>
@@ -6995,7 +6995,7 @@
       <c r="V71" t="inlineStr"/>
       <c r="W71" t="inlineStr"/>
       <c r="X71" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y71" t="b">
         <v>0</v>
@@ -7087,7 +7087,7 @@
       <c r="V72" t="inlineStr"/>
       <c r="W72" t="inlineStr"/>
       <c r="X72" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y72" t="b">
         <v>0</v>
@@ -7179,7 +7179,7 @@
       <c r="V73" t="inlineStr"/>
       <c r="W73" t="inlineStr"/>
       <c r="X73" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y73" t="b">
         <v>1</v>
@@ -7271,7 +7271,7 @@
       <c r="V74" t="inlineStr"/>
       <c r="W74" t="inlineStr"/>
       <c r="X74" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y74" t="b">
         <v>0</v>
@@ -7363,7 +7363,7 @@
       <c r="V75" t="inlineStr"/>
       <c r="W75" t="inlineStr"/>
       <c r="X75" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y75" t="b">
         <v>0</v>
@@ -7455,7 +7455,7 @@
       <c r="V76" t="inlineStr"/>
       <c r="W76" t="inlineStr"/>
       <c r="X76" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y76" t="b">
         <v>0</v>
@@ -7547,7 +7547,7 @@
       <c r="V77" t="inlineStr"/>
       <c r="W77" t="inlineStr"/>
       <c r="X77" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y77" t="b">
         <v>0</v>
@@ -7639,7 +7639,7 @@
       <c r="V78" t="inlineStr"/>
       <c r="W78" t="inlineStr"/>
       <c r="X78" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y78" t="b">
         <v>0</v>
@@ -7731,7 +7731,7 @@
       <c r="V79" t="inlineStr"/>
       <c r="W79" t="inlineStr"/>
       <c r="X79" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y79" t="b">
         <v>0</v>
@@ -7823,7 +7823,7 @@
       <c r="V80" t="inlineStr"/>
       <c r="W80" t="inlineStr"/>
       <c r="X80" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y80" t="b">
         <v>0</v>
@@ -7915,7 +7915,7 @@
       <c r="V81" t="inlineStr"/>
       <c r="W81" t="inlineStr"/>
       <c r="X81" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y81" t="b">
         <v>0</v>
@@ -8007,7 +8007,7 @@
       <c r="V82" t="inlineStr"/>
       <c r="W82" t="inlineStr"/>
       <c r="X82" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y82" t="b">
         <v>0</v>
@@ -8099,7 +8099,7 @@
       <c r="V83" t="inlineStr"/>
       <c r="W83" t="inlineStr"/>
       <c r="X83" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y83" t="b">
         <v>0</v>
@@ -8191,7 +8191,7 @@
       <c r="V84" t="inlineStr"/>
       <c r="W84" t="inlineStr"/>
       <c r="X84" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y84" t="b">
         <v>0</v>
@@ -8283,7 +8283,7 @@
       <c r="V85" t="inlineStr"/>
       <c r="W85" t="inlineStr"/>
       <c r="X85" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y85" t="b">
         <v>0</v>
@@ -8375,7 +8375,7 @@
       <c r="V86" t="inlineStr"/>
       <c r="W86" t="inlineStr"/>
       <c r="X86" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y86" t="b">
         <v>0</v>
@@ -8467,7 +8467,7 @@
       <c r="V87" t="inlineStr"/>
       <c r="W87" t="inlineStr"/>
       <c r="X87" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y87" t="b">
         <v>0</v>
@@ -8559,7 +8559,7 @@
       <c r="V88" t="inlineStr"/>
       <c r="W88" t="inlineStr"/>
       <c r="X88" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y88" t="b">
         <v>0</v>
@@ -8651,7 +8651,7 @@
       <c r="V89" t="inlineStr"/>
       <c r="W89" t="inlineStr"/>
       <c r="X89" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y89" t="b">
         <v>0</v>
@@ -8747,7 +8747,7 @@
       </c>
       <c r="W90" t="inlineStr"/>
       <c r="X90" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y90" t="b">
         <v>0</v>
@@ -8839,7 +8839,7 @@
       <c r="V91" t="inlineStr"/>
       <c r="W91" t="inlineStr"/>
       <c r="X91" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y91" t="b">
         <v>0</v>
@@ -8931,7 +8931,7 @@
       <c r="V92" t="inlineStr"/>
       <c r="W92" t="inlineStr"/>
       <c r="X92" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y92" t="b">
         <v>0</v>
@@ -9023,7 +9023,7 @@
       <c r="V93" t="inlineStr"/>
       <c r="W93" t="inlineStr"/>
       <c r="X93" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y93" t="b">
         <v>0</v>
@@ -9115,7 +9115,7 @@
       <c r="V94" t="inlineStr"/>
       <c r="W94" t="inlineStr"/>
       <c r="X94" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y94" t="b">
         <v>0</v>
@@ -9207,7 +9207,7 @@
       <c r="V95" t="inlineStr"/>
       <c r="W95" t="inlineStr"/>
       <c r="X95" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y95" t="b">
         <v>0</v>
@@ -9299,7 +9299,7 @@
       <c r="V96" t="inlineStr"/>
       <c r="W96" t="inlineStr"/>
       <c r="X96" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y96" t="b">
         <v>0</v>
@@ -9391,7 +9391,7 @@
       <c r="V97" t="inlineStr"/>
       <c r="W97" t="inlineStr"/>
       <c r="X97" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y97" t="b">
         <v>0</v>
@@ -9483,7 +9483,7 @@
       <c r="V98" t="inlineStr"/>
       <c r="W98" t="inlineStr"/>
       <c r="X98" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y98" t="b">
         <v>0</v>
@@ -9575,7 +9575,7 @@
       <c r="V99" t="inlineStr"/>
       <c r="W99" t="inlineStr"/>
       <c r="X99" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y99" t="b">
         <v>0</v>
@@ -9667,7 +9667,7 @@
       <c r="V100" t="inlineStr"/>
       <c r="W100" t="inlineStr"/>
       <c r="X100" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y100" t="b">
         <v>0</v>
@@ -9759,7 +9759,7 @@
       <c r="V101" t="inlineStr"/>
       <c r="W101" t="inlineStr"/>
       <c r="X101" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y101" t="b">
         <v>0</v>
@@ -9851,7 +9851,7 @@
       <c r="V102" t="inlineStr"/>
       <c r="W102" t="inlineStr"/>
       <c r="X102" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y102" t="b">
         <v>0</v>
@@ -9943,7 +9943,7 @@
       <c r="V103" t="inlineStr"/>
       <c r="W103" t="inlineStr"/>
       <c r="X103" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y103" t="b">
         <v>0</v>
@@ -10035,7 +10035,7 @@
       <c r="V104" t="inlineStr"/>
       <c r="W104" t="inlineStr"/>
       <c r="X104" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y104" t="b">
         <v>0</v>
@@ -10127,7 +10127,7 @@
       <c r="V105" t="inlineStr"/>
       <c r="W105" t="inlineStr"/>
       <c r="X105" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y105" t="b">
         <v>0</v>
@@ -10219,7 +10219,7 @@
       <c r="V106" t="inlineStr"/>
       <c r="W106" t="inlineStr"/>
       <c r="X106" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y106" t="b">
         <v>0</v>
@@ -10311,7 +10311,7 @@
       <c r="V107" t="inlineStr"/>
       <c r="W107" t="inlineStr"/>
       <c r="X107" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y107" t="b">
         <v>0</v>
@@ -10403,7 +10403,7 @@
       <c r="V108" t="inlineStr"/>
       <c r="W108" t="inlineStr"/>
       <c r="X108" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y108" t="b">
         <v>0</v>
@@ -10495,7 +10495,7 @@
       <c r="V109" t="inlineStr"/>
       <c r="W109" t="inlineStr"/>
       <c r="X109" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y109" t="b">
         <v>0</v>
@@ -10587,7 +10587,7 @@
         </is>
       </c>
       <c r="X110" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y110" t="b">
         <v>1</v>
@@ -10679,7 +10679,7 @@
         </is>
       </c>
       <c r="X111" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y111" t="b">
         <v>1</v>
@@ -10771,7 +10771,7 @@
       <c r="V112" t="inlineStr"/>
       <c r="W112" t="inlineStr"/>
       <c r="X112" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y112" t="b">
         <v>1</v>
@@ -10863,7 +10863,7 @@
         </is>
       </c>
       <c r="X113" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y113" t="b">
         <v>1</v>
@@ -10959,7 +10959,7 @@
         </is>
       </c>
       <c r="X114" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y114" t="b">
         <v>0</v>
@@ -11051,7 +11051,7 @@
       <c r="V115" t="inlineStr"/>
       <c r="W115" t="inlineStr"/>
       <c r="X115" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y115" t="b">
         <v>0</v>
@@ -11147,7 +11147,7 @@
         </is>
       </c>
       <c r="X116" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y116" t="b">
         <v>0</v>
@@ -11239,7 +11239,7 @@
       <c r="V117" t="inlineStr"/>
       <c r="W117" t="inlineStr"/>
       <c r="X117" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y117" t="b">
         <v>0</v>
@@ -11329,7 +11329,7 @@
         </is>
       </c>
       <c r="X118" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y118" t="b">
         <v>1</v>
@@ -11419,7 +11419,7 @@
         </is>
       </c>
       <c r="X119" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y119" t="b">
         <v>1</v>
@@ -11509,7 +11509,7 @@
         </is>
       </c>
       <c r="X120" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y120" t="b">
         <v>1</v>
@@ -11601,7 +11601,7 @@
       <c r="V121" t="inlineStr"/>
       <c r="W121" t="inlineStr"/>
       <c r="X121" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y121" t="b">
         <v>0</v>
@@ -11693,7 +11693,7 @@
       <c r="V122" t="inlineStr"/>
       <c r="W122" t="inlineStr"/>
       <c r="X122" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y122" t="b">
         <v>0</v>
@@ -11785,7 +11785,7 @@
       <c r="V123" t="inlineStr"/>
       <c r="W123" t="inlineStr"/>
       <c r="X123" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y123" t="b">
         <v>0</v>
@@ -11877,7 +11877,7 @@
       <c r="V124" t="inlineStr"/>
       <c r="W124" t="inlineStr"/>
       <c r="X124" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y124" t="b">
         <v>1</v>
@@ -11969,7 +11969,7 @@
       <c r="V125" t="inlineStr"/>
       <c r="W125" t="inlineStr"/>
       <c r="X125" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y125" t="b">
         <v>0</v>
@@ -12061,7 +12061,7 @@
       <c r="V126" t="inlineStr"/>
       <c r="W126" t="inlineStr"/>
       <c r="X126" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y126" t="b">
         <v>0</v>
@@ -12153,7 +12153,7 @@
       <c r="V127" t="inlineStr"/>
       <c r="W127" t="inlineStr"/>
       <c r="X127" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y127" t="b">
         <v>0</v>
@@ -12245,7 +12245,7 @@
       <c r="V128" t="inlineStr"/>
       <c r="W128" t="inlineStr"/>
       <c r="X128" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y128" t="b">
         <v>0</v>
@@ -12337,7 +12337,7 @@
       <c r="V129" t="inlineStr"/>
       <c r="W129" t="inlineStr"/>
       <c r="X129" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y129" t="b">
         <v>0</v>
@@ -12429,7 +12429,7 @@
       <c r="V130" t="inlineStr"/>
       <c r="W130" t="inlineStr"/>
       <c r="X130" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y130" t="b">
         <v>0</v>
@@ -12521,7 +12521,7 @@
       <c r="V131" t="inlineStr"/>
       <c r="W131" t="inlineStr"/>
       <c r="X131" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y131" t="b">
         <v>0</v>
@@ -12613,7 +12613,7 @@
       <c r="V132" t="inlineStr"/>
       <c r="W132" t="inlineStr"/>
       <c r="X132" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y132" t="b">
         <v>0</v>
@@ -12705,7 +12705,7 @@
       <c r="V133" t="inlineStr"/>
       <c r="W133" t="inlineStr"/>
       <c r="X133" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y133" t="b">
         <v>0</v>
@@ -12797,7 +12797,7 @@
       <c r="V134" t="inlineStr"/>
       <c r="W134" t="inlineStr"/>
       <c r="X134" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y134" t="b">
         <v>0</v>
@@ -12889,7 +12889,7 @@
       <c r="V135" t="inlineStr"/>
       <c r="W135" t="inlineStr"/>
       <c r="X135" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y135" t="b">
         <v>0</v>
@@ -12981,7 +12981,7 @@
       <c r="V136" t="inlineStr"/>
       <c r="W136" t="inlineStr"/>
       <c r="X136" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y136" t="b">
         <v>0</v>
@@ -13073,7 +13073,7 @@
       <c r="V137" t="inlineStr"/>
       <c r="W137" t="inlineStr"/>
       <c r="X137" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y137" t="b">
         <v>0</v>
@@ -13165,7 +13165,7 @@
       <c r="V138" t="inlineStr"/>
       <c r="W138" t="inlineStr"/>
       <c r="X138" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y138" t="b">
         <v>0</v>
@@ -13257,7 +13257,7 @@
       <c r="V139" t="inlineStr"/>
       <c r="W139" t="inlineStr"/>
       <c r="X139" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y139" t="b">
         <v>0</v>
@@ -13347,7 +13347,7 @@
       <c r="V140" t="inlineStr"/>
       <c r="W140" t="inlineStr"/>
       <c r="X140" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y140" t="b">
         <v>0</v>
@@ -13439,7 +13439,7 @@
       <c r="V141" t="inlineStr"/>
       <c r="W141" t="inlineStr"/>
       <c r="X141" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y141" t="b">
         <v>0</v>
@@ -13531,7 +13531,7 @@
       <c r="V142" t="inlineStr"/>
       <c r="W142" t="inlineStr"/>
       <c r="X142" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y142" t="b">
         <v>0</v>
@@ -13623,7 +13623,7 @@
       <c r="V143" t="inlineStr"/>
       <c r="W143" t="inlineStr"/>
       <c r="X143" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y143" t="b">
         <v>0</v>
@@ -13715,7 +13715,7 @@
       <c r="V144" t="inlineStr"/>
       <c r="W144" t="inlineStr"/>
       <c r="X144" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y144" t="b">
         <v>0</v>
@@ -13807,7 +13807,7 @@
       <c r="V145" t="inlineStr"/>
       <c r="W145" t="inlineStr"/>
       <c r="X145" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y145" t="b">
         <v>0</v>
@@ -13899,7 +13899,7 @@
       <c r="V146" t="inlineStr"/>
       <c r="W146" t="inlineStr"/>
       <c r="X146" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y146" t="b">
         <v>0</v>
@@ -13991,7 +13991,7 @@
       <c r="V147" t="inlineStr"/>
       <c r="W147" t="inlineStr"/>
       <c r="X147" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y147" t="b">
         <v>0</v>
@@ -14083,7 +14083,7 @@
       <c r="V148" t="inlineStr"/>
       <c r="W148" t="inlineStr"/>
       <c r="X148" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y148" t="b">
         <v>0</v>
@@ -14175,7 +14175,7 @@
       <c r="V149" t="inlineStr"/>
       <c r="W149" t="inlineStr"/>
       <c r="X149" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y149" t="b">
         <v>0</v>
@@ -14267,7 +14267,7 @@
       <c r="V150" t="inlineStr"/>
       <c r="W150" t="inlineStr"/>
       <c r="X150" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y150" t="b">
         <v>0</v>
@@ -14359,7 +14359,7 @@
       <c r="V151" t="inlineStr"/>
       <c r="W151" t="inlineStr"/>
       <c r="X151" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y151" t="b">
         <v>0</v>
@@ -14451,7 +14451,7 @@
       <c r="V152" t="inlineStr"/>
       <c r="W152" t="inlineStr"/>
       <c r="X152" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y152" t="b">
         <v>0</v>
@@ -14543,7 +14543,7 @@
       <c r="V153" t="inlineStr"/>
       <c r="W153" t="inlineStr"/>
       <c r="X153" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y153" t="b">
         <v>0</v>
@@ -14635,7 +14635,7 @@
       <c r="V154" t="inlineStr"/>
       <c r="W154" t="inlineStr"/>
       <c r="X154" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y154" t="b">
         <v>0</v>
@@ -14727,7 +14727,7 @@
       <c r="V155" t="inlineStr"/>
       <c r="W155" t="inlineStr"/>
       <c r="X155" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y155" t="b">
         <v>0</v>
@@ -14819,7 +14819,7 @@
       <c r="V156" t="inlineStr"/>
       <c r="W156" t="inlineStr"/>
       <c r="X156" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y156" t="b">
         <v>0</v>
@@ -14911,7 +14911,7 @@
       <c r="V157" t="inlineStr"/>
       <c r="W157" t="inlineStr"/>
       <c r="X157" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y157" t="b">
         <v>0</v>
@@ -15003,7 +15003,7 @@
       <c r="V158" t="inlineStr"/>
       <c r="W158" t="inlineStr"/>
       <c r="X158" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y158" t="b">
         <v>0</v>
@@ -15095,7 +15095,7 @@
       <c r="V159" t="inlineStr"/>
       <c r="W159" t="inlineStr"/>
       <c r="X159" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y159" t="b">
         <v>0</v>
@@ -15183,7 +15183,7 @@
         </is>
       </c>
       <c r="X160" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y160" t="b">
         <v>1</v>
@@ -15275,7 +15275,7 @@
       <c r="V161" t="inlineStr"/>
       <c r="W161" t="inlineStr"/>
       <c r="X161" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y161" t="b">
         <v>0</v>
@@ -15367,7 +15367,7 @@
       <c r="V162" t="inlineStr"/>
       <c r="W162" t="inlineStr"/>
       <c r="X162" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y162" t="b">
         <v>0</v>
@@ -15459,7 +15459,7 @@
       <c r="V163" t="inlineStr"/>
       <c r="W163" t="inlineStr"/>
       <c r="X163" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y163" t="b">
         <v>0</v>
@@ -15551,7 +15551,7 @@
       <c r="V164" t="inlineStr"/>
       <c r="W164" t="inlineStr"/>
       <c r="X164" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y164" t="b">
         <v>0</v>
@@ -15643,7 +15643,7 @@
       <c r="V165" t="inlineStr"/>
       <c r="W165" t="inlineStr"/>
       <c r="X165" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y165" t="b">
         <v>0</v>
@@ -15735,7 +15735,7 @@
       <c r="V166" t="inlineStr"/>
       <c r="W166" t="inlineStr"/>
       <c r="X166" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y166" t="b">
         <v>0</v>
@@ -15827,7 +15827,7 @@
       <c r="V167" t="inlineStr"/>
       <c r="W167" t="inlineStr"/>
       <c r="X167" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y167" t="b">
         <v>0</v>
@@ -15919,7 +15919,7 @@
       <c r="V168" t="inlineStr"/>
       <c r="W168" t="inlineStr"/>
       <c r="X168" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y168" t="b">
         <v>0</v>
@@ -16011,7 +16011,7 @@
       <c r="V169" t="inlineStr"/>
       <c r="W169" t="inlineStr"/>
       <c r="X169" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y169" t="b">
         <v>0</v>
@@ -16103,7 +16103,7 @@
       <c r="V170" t="inlineStr"/>
       <c r="W170" t="inlineStr"/>
       <c r="X170" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y170" t="b">
         <v>0</v>
@@ -16195,7 +16195,7 @@
       <c r="V171" t="inlineStr"/>
       <c r="W171" t="inlineStr"/>
       <c r="X171" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y171" t="b">
         <v>0</v>
@@ -16287,7 +16287,7 @@
       <c r="V172" t="inlineStr"/>
       <c r="W172" t="inlineStr"/>
       <c r="X172" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y172" t="b">
         <v>0</v>
@@ -16379,7 +16379,7 @@
       <c r="V173" t="inlineStr"/>
       <c r="W173" t="inlineStr"/>
       <c r="X173" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y173" t="b">
         <v>1</v>
@@ -16471,7 +16471,7 @@
       <c r="V174" t="inlineStr"/>
       <c r="W174" t="inlineStr"/>
       <c r="X174" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y174" t="b">
         <v>0</v>
@@ -16563,7 +16563,7 @@
       <c r="V175" t="inlineStr"/>
       <c r="W175" t="inlineStr"/>
       <c r="X175" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y175" t="b">
         <v>0</v>
@@ -16655,7 +16655,7 @@
       <c r="V176" t="inlineStr"/>
       <c r="W176" t="inlineStr"/>
       <c r="X176" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y176" t="b">
         <v>0</v>
@@ -16747,7 +16747,7 @@
       <c r="V177" t="inlineStr"/>
       <c r="W177" t="inlineStr"/>
       <c r="X177" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y177" t="b">
         <v>0</v>
@@ -16839,7 +16839,7 @@
       <c r="V178" t="inlineStr"/>
       <c r="W178" t="inlineStr"/>
       <c r="X178" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y178" t="b">
         <v>0</v>
@@ -16931,7 +16931,7 @@
       <c r="V179" t="inlineStr"/>
       <c r="W179" t="inlineStr"/>
       <c r="X179" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y179" t="b">
         <v>0</v>
@@ -17023,7 +17023,7 @@
       <c r="V180" t="inlineStr"/>
       <c r="W180" t="inlineStr"/>
       <c r="X180" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y180" t="b">
         <v>0</v>
@@ -17115,7 +17115,7 @@
       <c r="V181" t="inlineStr"/>
       <c r="W181" t="inlineStr"/>
       <c r="X181" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y181" t="b">
         <v>0</v>
@@ -17207,7 +17207,7 @@
       <c r="V182" t="inlineStr"/>
       <c r="W182" t="inlineStr"/>
       <c r="X182" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y182" t="b">
         <v>0</v>
@@ -17299,7 +17299,7 @@
       <c r="V183" t="inlineStr"/>
       <c r="W183" t="inlineStr"/>
       <c r="X183" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y183" t="b">
         <v>0</v>
@@ -17391,7 +17391,7 @@
         </is>
       </c>
       <c r="X184" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y184" t="b">
         <v>0</v>
@@ -17483,7 +17483,7 @@
       <c r="V185" t="inlineStr"/>
       <c r="W185" t="inlineStr"/>
       <c r="X185" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y185" t="b">
         <v>0</v>
@@ -17575,7 +17575,7 @@
       <c r="V186" t="inlineStr"/>
       <c r="W186" t="inlineStr"/>
       <c r="X186" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y186" t="b">
         <v>0</v>
@@ -17667,7 +17667,7 @@
       <c r="V187" t="inlineStr"/>
       <c r="W187" t="inlineStr"/>
       <c r="X187" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y187" t="b">
         <v>0</v>
@@ -17759,7 +17759,7 @@
       <c r="V188" t="inlineStr"/>
       <c r="W188" t="inlineStr"/>
       <c r="X188" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y188" t="b">
         <v>0</v>
@@ -17857,7 +17857,7 @@
         </is>
       </c>
       <c r="X189" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y189" t="b">
         <v>0</v>
@@ -17955,7 +17955,7 @@
         </is>
       </c>
       <c r="X190" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y190" t="b">
         <v>0</v>
@@ -18047,7 +18047,7 @@
       <c r="V191" t="inlineStr"/>
       <c r="W191" t="inlineStr"/>
       <c r="X191" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y191" t="b">
         <v>0</v>
@@ -18139,7 +18139,7 @@
       <c r="V192" t="inlineStr"/>
       <c r="W192" t="inlineStr"/>
       <c r="X192" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y192" t="b">
         <v>0</v>
@@ -18231,7 +18231,7 @@
       <c r="V193" t="inlineStr"/>
       <c r="W193" t="inlineStr"/>
       <c r="X193" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y193" t="b">
         <v>0</v>
@@ -18323,7 +18323,7 @@
       <c r="V194" t="inlineStr"/>
       <c r="W194" t="inlineStr"/>
       <c r="X194" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y194" t="b">
         <v>0</v>
@@ -18421,7 +18421,7 @@
         </is>
       </c>
       <c r="X195" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y195" t="b">
         <v>0</v>
@@ -18513,7 +18513,7 @@
       <c r="V196" t="inlineStr"/>
       <c r="W196" t="inlineStr"/>
       <c r="X196" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y196" t="b">
         <v>0</v>
@@ -18605,7 +18605,7 @@
       <c r="V197" t="inlineStr"/>
       <c r="W197" t="inlineStr"/>
       <c r="X197" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y197" t="b">
         <v>0</v>
@@ -18703,7 +18703,7 @@
         </is>
       </c>
       <c r="X198" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y198" t="b">
         <v>0</v>
@@ -18795,7 +18795,7 @@
       <c r="V199" t="inlineStr"/>
       <c r="W199" t="inlineStr"/>
       <c r="X199" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y199" t="b">
         <v>0</v>
@@ -18887,7 +18887,7 @@
       <c r="V200" t="inlineStr"/>
       <c r="W200" t="inlineStr"/>
       <c r="X200" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y200" t="b">
         <v>0</v>
@@ -18985,7 +18985,7 @@
         </is>
       </c>
       <c r="X201" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y201" t="b">
         <v>0</v>
@@ -19083,7 +19083,7 @@
         </is>
       </c>
       <c r="X202" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y202" t="b">
         <v>0</v>
@@ -19175,7 +19175,7 @@
       <c r="V203" t="inlineStr"/>
       <c r="W203" t="inlineStr"/>
       <c r="X203" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y203" t="b">
         <v>0</v>
@@ -19267,7 +19267,7 @@
       <c r="V204" t="inlineStr"/>
       <c r="W204" t="inlineStr"/>
       <c r="X204" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y204" t="b">
         <v>0</v>
@@ -19359,7 +19359,7 @@
       <c r="V205" t="inlineStr"/>
       <c r="W205" t="inlineStr"/>
       <c r="X205" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y205" t="b">
         <v>0</v>
@@ -19451,7 +19451,7 @@
       <c r="V206" t="inlineStr"/>
       <c r="W206" t="inlineStr"/>
       <c r="X206" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y206" t="b">
         <v>0</v>
@@ -19543,7 +19543,7 @@
       <c r="V207" t="inlineStr"/>
       <c r="W207" t="inlineStr"/>
       <c r="X207" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y207" t="b">
         <v>0</v>
@@ -19635,7 +19635,7 @@
       <c r="V208" t="inlineStr"/>
       <c r="W208" t="inlineStr"/>
       <c r="X208" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y208" t="b">
         <v>0</v>
@@ -19727,7 +19727,7 @@
       <c r="V209" t="inlineStr"/>
       <c r="W209" t="inlineStr"/>
       <c r="X209" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y209" t="b">
         <v>1</v>
@@ -19819,7 +19819,7 @@
       <c r="V210" t="inlineStr"/>
       <c r="W210" t="inlineStr"/>
       <c r="X210" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y210" t="b">
         <v>1</v>
@@ -19911,7 +19911,7 @@
       <c r="V211" t="inlineStr"/>
       <c r="W211" t="inlineStr"/>
       <c r="X211" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y211" t="b">
         <v>1</v>
@@ -20003,7 +20003,7 @@
       <c r="V212" t="inlineStr"/>
       <c r="W212" t="inlineStr"/>
       <c r="X212" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y212" t="b">
         <v>0</v>
@@ -20095,7 +20095,7 @@
       <c r="V213" t="inlineStr"/>
       <c r="W213" t="inlineStr"/>
       <c r="X213" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y213" t="b">
         <v>0</v>
@@ -20187,7 +20187,7 @@
       <c r="V214" t="inlineStr"/>
       <c r="W214" t="inlineStr"/>
       <c r="X214" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y214" t="b">
         <v>0</v>
@@ -20279,7 +20279,7 @@
       <c r="V215" t="inlineStr"/>
       <c r="W215" t="inlineStr"/>
       <c r="X215" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y215" t="b">
         <v>0</v>
@@ -20371,7 +20371,7 @@
       <c r="V216" t="inlineStr"/>
       <c r="W216" t="inlineStr"/>
       <c r="X216" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y216" t="b">
         <v>0</v>
@@ -20463,7 +20463,7 @@
       <c r="V217" t="inlineStr"/>
       <c r="W217" t="inlineStr"/>
       <c r="X217" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y217" t="b">
         <v>0</v>
@@ -20555,7 +20555,7 @@
       <c r="V218" t="inlineStr"/>
       <c r="W218" t="inlineStr"/>
       <c r="X218" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y218" t="b">
         <v>0</v>
@@ -20647,7 +20647,7 @@
       <c r="V219" t="inlineStr"/>
       <c r="W219" t="inlineStr"/>
       <c r="X219" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y219" t="b">
         <v>0</v>
@@ -20743,7 +20743,7 @@
         </is>
       </c>
       <c r="X220" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y220" t="b">
         <v>0</v>
@@ -20835,7 +20835,7 @@
       <c r="V221" t="inlineStr"/>
       <c r="W221" t="inlineStr"/>
       <c r="X221" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y221" t="b">
         <v>0</v>
@@ -20927,7 +20927,7 @@
       <c r="V222" t="inlineStr"/>
       <c r="W222" t="inlineStr"/>
       <c r="X222" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y222" t="b">
         <v>0</v>
@@ -21019,7 +21019,7 @@
       <c r="V223" t="inlineStr"/>
       <c r="W223" t="inlineStr"/>
       <c r="X223" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y223" t="b">
         <v>0</v>
@@ -21115,7 +21115,7 @@
         </is>
       </c>
       <c r="X224" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y224" t="b">
         <v>0</v>
@@ -21207,7 +21207,7 @@
       <c r="V225" t="inlineStr"/>
       <c r="W225" t="inlineStr"/>
       <c r="X225" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y225" t="b">
         <v>0</v>
@@ -21299,7 +21299,7 @@
       <c r="V226" t="inlineStr"/>
       <c r="W226" t="inlineStr"/>
       <c r="X226" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y226" t="b">
         <v>0</v>
@@ -21391,7 +21391,7 @@
       <c r="V227" t="inlineStr"/>
       <c r="W227" t="inlineStr"/>
       <c r="X227" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y227" t="b">
         <v>0</v>
@@ -21483,7 +21483,7 @@
       <c r="V228" t="inlineStr"/>
       <c r="W228" t="inlineStr"/>
       <c r="X228" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y228" t="b">
         <v>0</v>
@@ -21571,7 +21571,7 @@
       </c>
       <c r="W229" t="inlineStr"/>
       <c r="X229" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y229" t="b">
         <v>1</v>
@@ -21659,7 +21659,7 @@
       <c r="V230" t="inlineStr"/>
       <c r="W230" t="inlineStr"/>
       <c r="X230" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y230" t="b">
         <v>0</v>
@@ -21755,7 +21755,7 @@
       </c>
       <c r="W231" t="inlineStr"/>
       <c r="X231" s="2" t="n">
-        <v>46290.83268518518</v>
+        <v>46293.32679398148</v>
       </c>
       <c r="Y231" t="b">
         <v>0</v>

</xml_diff>